<commit_message>
feat: rerank-2.5, knee-point filter, eval recursive context fix, MongoDB TLS
- Wire config.VOYAGE_RERANK_MODEL in voyage.py (was hardcoded 'rerank-2');
  set VOYAGE_RERANK_MODEL=rerank-2.5 in .env
- Add knee_filter() to voyage.py: absolute-gap primary (>0.15), largest-gap
  fallback (>0.05 noise floor), min 2 chunks; gated by RERANK_KNEE_ENABLED
- Fix run_pipeline_eval to return deduped anchor+followup chunks for recursive
  queries — RAGAS context was missing the anchor pass entirely
- Fix MongoClient tlsAllowInvalidCertificates=True (Python 3.14 / OpenSSL
  3.5.5 TLS handshake regression)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tamu_data/evals/golden_sets/golden_20260313_draft_v1.xlsx
+++ b/tamu_data/evals/golden_sets/golden_20260313_draft_v1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1667,33 +1667,31 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>What courses would you recommend taking after CSCE 632 to continue learning about HCl concepts?</t>
+          <t>How do I set up a React project from scratch?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Assignments are designed to help you engage with HCl concepts. Doing anything to
-subvert the learning objectives harm your learning experience and constitute
-academic dishonesty.</t>
+          <t>(out of scope)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>recurrent</t>
+          <t>out_of_scope</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>How do I set up a React project from scratch?</t>
+          <t>Can you write a Python function to sort a list?</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1709,11 +1707,11 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Can you write a Python function to sort a list?</t>
+          <t>Who won the Super Bowl last year?</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1722,26 +1720,6 @@
         </is>
       </c>
       <c r="D51" t="inlineStr">
-        <is>
-          <t>out_of_scope</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Who won the Super Bowl last year?</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>(out of scope)</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
         <is>
           <t>out_of_scope</t>
         </is>

</xml_diff>